<commit_message>
Stage 1 smoke-test passed: end-to-end works
- Migration 002 seeds basic expense/income categories (food, transport, cafe, ...)
- sync.py made resilient: unknown account/category/currency does not throw
  FK errors anymore — values default to NULL and original ID is recorded in
  note with [unresolved: ...] tag for manual reconciliation later.

Verified flow:
  Telegram message "25 EUR food тест"
    → finance_stepan_bot
    → Cloudflare Worker /tg
    → D1 expenses_outbox
    → sync.py pulled 1, inserted 1, confirmed 1
    → local SQLite expenses row
    → regenerated Finances.generated.xlsx

Stage 1 complete.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/finances/Finances.generated.xlsx
+++ b/finances/Finances.generated.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>id</t>
   </si>
@@ -76,6 +76,21 @@
   </si>
   <si>
     <t>created_at</t>
+  </si>
+  <si>
+    <t>2026-05-23</t>
+  </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>тест</t>
+  </si>
+  <si>
+    <t>telegram</t>
+  </si>
+  <si>
+    <t>2026-05-23T14:48:03.933Z</t>
   </si>
   <si>
     <t>base</t>
@@ -481,7 +496,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -508,6 +523,29 @@
       </c>
       <c r="H1" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -525,19 +563,19 @@
         <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E1" t="s">
         <v>18</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>